<commit_message>
Predložak ugovora A.02 potpuno izmišljen: stavke PR-1 do PR-3 s opisima primjera, izmišljene pozicije i naslovi, napomena u radnoj knjizi; test pazi da stavke ostanu označene kao primjer
</commit_message>
<xml_diff>
--- a/docs/predlosci/odrzavanje/ugovor-a02.xlsx
+++ b/docs/predlosci/odrzavanje/ugovor-a02.xlsx
@@ -72,6 +72,18 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Napomena:</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izmišljeni primjer oblika za goCOP. Nije ugovor ni troškovnik Hrvatskih voda.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -94,7 +106,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A.02.01.01.01.01.01.</t>
+          <t xml:space="preserve">A.02.01.01.01.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -159,7 +171,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.6. Uklanjanje vegetacije</t>
+          <t xml:space="preserve">Primjer vrste usluge</t>
         </is>
       </c>
     </row>
@@ -202,12 +214,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strojna košnja trave na ravnim površinama</t>
+          <t xml:space="preserve">Primjer stavke: košnja trave (izmišljeno)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">225</t>
+          <t xml:space="preserve">PR-1</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -244,12 +256,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strojna košnja trave na kosim površinama</t>
+          <t xml:space="preserve">Primjer stavke: košnja pokosa (izmišljeno)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t xml:space="preserve">226</t>
+          <t xml:space="preserve">PR-2</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -288,7 +300,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t xml:space="preserve">A.02.01.01.02.04.</t>
+          <t xml:space="preserve">A.02.01.01.02.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -353,7 +365,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.6. Uklanjanje vegetacije</t>
+          <t xml:space="preserve">Primjer vrste usluge</t>
         </is>
       </c>
     </row>
@@ -396,12 +408,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strojno odstranjivanje šaša i trske</t>
+          <t xml:space="preserve">Primjer stavke: uklanjanje trske (izmišljeno)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t xml:space="preserve">229</t>
+          <t xml:space="preserve">PR-3</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -442,7 +454,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">POPIS LOKACIJA IZVRŠENJA USLUGA</t>
+          <t xml:space="preserve">POPIS LOKACIJA — IZMIŠLJENI PRIMJER</t>
         </is>
       </c>
     </row>
@@ -450,31 +462,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">RED VODE</t>
+          <t xml:space="preserve">Red vode</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VRSTA VODE</t>
+          <t xml:space="preserve">Vrsta</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAZIV VODE</t>
+          <t xml:space="preserve">Naziv</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VODE I. REDA - Ostale državne vode</t>
+          <t xml:space="preserve">VODE I. REDA - ostale državne vode (primjer)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Vodotoci</t>
+          <t xml:space="preserve">1. Vodotoci (primjer)</t>
         </is>
       </c>
     </row>
@@ -493,14 +505,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">VODE II. REDA</t>
+          <t xml:space="preserve">VODE II. REDA (primjer)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. Osnovne melioracijske građevine za odvodnju</t>
+          <t xml:space="preserve">4. Melioracijski kanali (primjer)</t>
         </is>
       </c>
     </row>
@@ -551,12 +563,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">225</t>
+          <t xml:space="preserve">PR-1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strojna košnja trave na ravnim površinama</t>
+          <t xml:space="preserve">Primjer stavke: košnja trave (izmišljeno)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -571,12 +583,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">226</t>
+          <t xml:space="preserve">PR-2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strojna košnja trave na kosim površinama</t>
+          <t xml:space="preserve">Primjer stavke: košnja pokosa (izmišljeno)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -591,12 +603,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">229</t>
+          <t xml:space="preserve">PR-3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strojno odstranjivanje šaša i trske</t>
+          <t xml:space="preserve">Primjer stavke: uklanjanje trske (izmišljeno)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>